<commit_message>
etapa 01 - final
</commit_message>
<xml_diff>
--- a/Datasetsd.xlsx
+++ b/Datasetsd.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8845de8732abbeb5/Documentos/GitHub/trabalhoMLmsc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3129827-F354-4FB1-913F-3B526711EAFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{E3129827-F354-4FB1-913F-3B526711EAFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A25E0AC-1BB7-40D0-AE5C-96873E5B7CFA}"/>
   <bookViews>
-    <workbookView xWindow="5320" yWindow="3120" windowWidth="14310" windowHeight="7300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="35055" yWindow="5340" windowWidth="14235" windowHeight="7275" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -143,7 +143,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -160,6 +160,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -882,7 +883,7 @@
             <c:numRef>
               <c:f>Sheet1!$B$9:$B$10</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>144.80000000000001</c:v>
@@ -1002,7 +1003,7 @@
             <c:numRef>
               <c:f>Sheet1!$C$9:$C$10</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>36.200000000000003</c:v>
@@ -1105,7 +1106,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1400,7 +1401,7 @@
             <c:numRef>
               <c:f>Sheet1!$B$14:$B$15</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>544.80000000000007</c:v>
@@ -1520,7 +1521,7 @@
             <c:numRef>
               <c:f>Sheet1!$C$14:$C$15</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>136.20000000000002</c:v>
@@ -1623,7 +1624,7 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="0" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -4799,11 +4800,11 @@
       <c r="A9" t="s">
         <v>0</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="6">
         <f>$D$9*80%</f>
         <v>144.80000000000001</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="6">
         <f>$D$9*20%</f>
         <v>36.200000000000003</v>
       </c>
@@ -4815,11 +4816,11 @@
       <c r="A10" t="s">
         <v>1</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="6">
         <f>$D$10*80%</f>
         <v>134.4</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="6">
         <f>$D$10*20%</f>
         <v>33.6</v>
       </c>
@@ -4845,11 +4846,11 @@
       <c r="A14" t="s">
         <v>0</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="6">
         <f>D14*80%</f>
         <v>544.80000000000007</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="6">
         <f>D14*20%</f>
         <v>136.20000000000002</v>
       </c>
@@ -4861,11 +4862,11 @@
       <c r="A15" t="s">
         <v>1</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="6">
         <f>D15*80%</f>
         <v>534.4</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="6">
         <f>D15*20%</f>
         <v>133.6</v>
       </c>

</xml_diff>